<commit_message>
build: GST-001 — lift header_row_style import + extract Local Guide sample data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book.xlsx
+++ b/templates/_masters/GST-001-welcome-book.xlsx
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -205,6 +205,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1255,22 +1258,22 @@
           <t>Coffee</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Mountain Grind</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>0.8 mi</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>(865) 555-0100</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Best espresso in town; small pastry case fills fast</t>
         </is>
@@ -1282,10 +1285,10 @@
           <t>Coffee</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1293,22 +1296,22 @@
           <t>Restaurant</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>The Cast Iron</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>2.1 mi</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>(865) 555-0118</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Sunday brunch is chef's-kiss — reserve ahead</t>
         </is>
@@ -1320,22 +1323,22 @@
           <t>Restaurant</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Ridge BBQ</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>1.4 mi</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>(865) 555-0122</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Brisket sells out by 7 PM Fri/Sat</t>
         </is>
@@ -1347,10 +1350,10 @@
           <t>Restaurant</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -1358,10 +1361,10 @@
           <t>Grocery</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr"/>
-      <c r="E11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1369,10 +1372,10 @@
           <t>Grocery</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr"/>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -1380,10 +1383,10 @@
           <t>Takeout</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr"/>
-      <c r="E13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1391,10 +1394,10 @@
           <t>Takeout</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -1402,10 +1405,10 @@
           <t>Pharmacy</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr"/>
-      <c r="E15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1413,10 +1416,10 @@
           <t>Gas station</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -1424,10 +1427,10 @@
           <t>Hospital/Urgent care</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -1435,10 +1438,10 @@
           <t>Coffee alt</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -1446,10 +1449,10 @@
           <t>Outdoor/Hike</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1457,10 +1460,10 @@
           <t>Outdoor/Hike</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -1468,10 +1471,10 @@
           <t>Kid-friendly</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -1479,10 +1482,10 @@
           <t>Kid-friendly</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -1490,10 +1493,10 @@
           <t>Date night</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -1501,10 +1504,10 @@
           <t>Bar/Nightlife</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
@@ -1512,10 +1515,10 @@
           <t>Emergency (non-911)</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1704,13 +1707,13 @@
           <t>Checkout day:</t>
         </is>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="15">
         <f>IF(Welcome!B9&lt;&gt;"", TEXT(Welcome!B9,"dddd, mmmm d"), "See Welcome tab")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Before you leave — please:</t>
         </is>
@@ -1834,7 +1837,7 @@
     </row>
     <row r="4" ht="12" customHeight="1"/>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>IN AN EMERGENCY — CALL 911</t>
         </is>
@@ -1955,7 +1958,7 @@
           <t>Host phone (call/text):</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="15">
         <f>Welcome!B7</f>
         <v/>
       </c>
@@ -2127,7 +2130,7 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>⚠ RIGHT-CLICK this tab → Hide before sharing the workbook or exporting to PDF.</t>
         </is>

</xml_diff>